<commit_message>
Allure reports and tweaks
</commit_message>
<xml_diff>
--- a/Selenium_BestBuy/data/testdata.xlsx
+++ b/Selenium_BestBuy/data/testdata.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Wipro_Capstone\Selenium_BestBuy\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{781CB7A2-B583-47C2-B42D-D9EF3CDF135F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43839A3E-1B22-43D6-80A5-95E7B6DAD31D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PositiveData" sheetId="1" r:id="rId1"/>
     <sheet name="NegativeData" sheetId="2" r:id="rId2"/>
+    <sheet name="CheckoutNegativeData" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="22">
   <si>
     <t>TC_ID</t>
   </si>
@@ -80,6 +81,18 @@
   </si>
   <si>
     <t>UnsupportedFilter</t>
+  </si>
+  <si>
+    <t>TC_07</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>InvalidCheckoutEmail</t>
+  </si>
+  <si>
+    <t>abc123#67</t>
   </si>
 </sst>
 </file>
@@ -525,4 +538,40 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CC89AA9-1E4F-44C7-9C26-90AE6E0E525B}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="18.5703125" customWidth="1"/>
+    <col min="3" max="3" width="22.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>